<commit_message>
Corregimos el excel de la dimensión social
</commit_message>
<xml_diff>
--- a/data/processed/indicadores_SOC_SIEPAC.xlsx
+++ b/data/processed/indicadores_SOC_SIEPAC.xlsx
@@ -985,19 +985,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0.001674700183943291</v>
+        <v>1.674700183943275</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.001704469904945673</v>
+        <v>1.704469904945673</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.001676745166674422</v>
+        <v>1.676745166674422</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0.00169191796099463</v>
+        <v>1.69191796099463</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.001701856994641966</v>
+        <v>1.701856994641966</v>
       </c>
     </row>
     <row r="7">
@@ -1029,19 +1029,19 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>3.629698996419138</v>
+        <v>8.711277591405931</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>3.029175503007524</v>
+        <v>7.270021207218058</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>2.95066870659458</v>
+        <v>7.08160489582699</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2.535527284910263</v>
+        <v>6.085265483784632</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>2.214336134299205</v>
+        <v>5.314406722318093</v>
       </c>
     </row>
     <row r="9">
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>3.290942100000229</v>
+        <v>4.416709446457916</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>3.065208624391028</v>
+        <v>4.055810480932906</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3.106351586979381</v>
+        <v>4.074019022102741</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3.032350310461753</v>
+        <v>3.905677684113087</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>3.091759270974054</v>
+        <v>3.891796891918423</v>
       </c>
     </row>
   </sheetData>
@@ -1197,19 +1197,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0.006225959217700948</v>
+        <v>6.22595921770089</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.006336632800148852</v>
+        <v>6.336632800148852</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.006233561760058678</v>
+        <v>6.233561760058678</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0.006289968990177774</v>
+        <v>6.289968990177773</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.006326918898432973</v>
+        <v>6.326918898432972</v>
       </c>
     </row>
     <row r="7">
@@ -1241,19 +1241,19 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>9.497326752261355</v>
+        <v>22.79360082023156</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>7.926020744527325</v>
+        <v>19.02246365279723</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>7.720602967862492</v>
+        <v>18.52946062943986</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>6.634360352696893</v>
+        <v>15.9224764527489</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>5.793944298831981</v>
+        <v>13.90547645323327</v>
       </c>
     </row>
     <row r="9">
@@ -1285,19 +1285,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>22.23950903338138</v>
+        <v>25.49217692112361</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>21.16114533575594</v>
+        <v>24.06560184835905</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>22.61410963655608</v>
+        <v>25.45347394653541</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>22.57852348242082</v>
+        <v>25.17382266929409</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>24.68762740427068</v>
+        <v>27.09298142659333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregimos datos en la dimension social, SOC2 ES
</commit_message>
<xml_diff>
--- a/data/processed/indicadores_SOC_SIEPAC.xlsx
+++ b/data/processed/indicadores_SOC_SIEPAC.xlsx
@@ -963,19 +963,19 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>6.18992678570214</v>
+        <v>2.063308928567357</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>6.093497221687183</v>
+        <v>2.031165740562394</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>5.595099691236247</v>
+        <v>1.865033230412082</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>5.1863096066683</v>
+        <v>1.728769868889434</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>5.278357503398404</v>
+        <v>1.759452501132801</v>
       </c>
     </row>
     <row r="6">
@@ -1051,19 +1051,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>2.416622630946807</v>
+        <v>0.8055408769822704</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2.252187570882236</v>
+        <v>0.7507291902940787</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>2.400984229520648</v>
+        <v>0.8003280765068828</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2.346501664381798</v>
+        <v>0.7821672214605995</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2.61879044419974</v>
+        <v>0.8729301480665801</v>
       </c>
     </row>
     <row r="10">
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>4.416709446457916</v>
+        <v>3.460426177941363</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>4.055810480932906</v>
+        <v>3.128512170647415</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>4.074019022102741</v>
+        <v>3.185565253129752</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3.905677684113087</v>
+        <v>3.068698653996409</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>3.891796891918423</v>
+        <v>3.014336008851963</v>
       </c>
     </row>
   </sheetData>
@@ -1175,19 +1175,19 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>21.72650072973297</v>
+        <v>7.2421669099111</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>22.66387232801</v>
+        <v>7.554624109336666</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>21.026279414898</v>
+        <v>7.008759804965998</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>20.74355638031428</v>
+        <v>6.914518793438093</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>21.70361037554047</v>
+        <v>7.234536791846826</v>
       </c>
     </row>
     <row r="6">
@@ -1263,19 +1263,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>31.40490513181162</v>
+        <v>10.4683017106039</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>29.27843752653015</v>
+        <v>9.759479175510052</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>30.37673705619569</v>
+        <v>10.1255790187319</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>26.87122889154614</v>
+        <v>8.957076297182045</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>33.15575667431635</v>
+        <v>11.05191889143878</v>
       </c>
     </row>
     <row r="10">
@@ -1285,19 +1285,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>25.49217692112361</v>
+        <v>19.58868738095201</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>24.06560184835905</v>
+        <v>18.29423408674348</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>25.45347394653541</v>
+        <v>19.74202767196945</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>25.17382266929409</v>
+        <v>19.88329097242071</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>27.09298142659333</v>
+        <v>20.99749619883145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregimos datos en SOCs - SOC2 PAN
</commit_message>
<xml_diff>
--- a/data/processed/indicadores_SOC_SIEPAC.xlsx
+++ b/data/processed/indicadores_SOC_SIEPAC.xlsx
@@ -729,19 +729,19 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
     </row>
     <row r="5">
@@ -751,19 +751,19 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>2.200000000000003</v>
+        <v>2.2</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>2.099999999999994</v>
+        <v>2.09999999999999</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>1.799999999999997</v>
+        <v>1.8</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1.700000000000003</v>
+        <v>1.7</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1.700000000000003</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="6">
@@ -773,10 +773,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>10.09999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>10.73999999999999</v>
+        <v>10.74</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>10.06</v>
@@ -820,16 +820,16 @@
         <v>1.5</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>0.9099999999999966</v>
+        <v>0.909999999999997</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.7399999999999949</v>
+        <v>0.739999999999995</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>0.5900000000000034</v>
+        <v>0.590000000000003</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>0.4429999999999978</v>
+        <v>0.442999999999998</v>
       </c>
     </row>
     <row r="9">
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>5.599999999999994</v>
+        <v>5.59999999999999</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>5.099999999999994</v>
+        <v>5.09999999999999</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>4.799999999999997</v>
+        <v>4.8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4.400000000000006</v>
+        <v>4.40000000000001</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>4</v>
@@ -861,13 +861,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>5.796666666666664</v>
+        <v>5.796666666666663</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>5.61333333333333</v>
+        <v>5.613333333333329</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>5.394999999999999</v>
+        <v>5.394999999999997</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>5.103333333333334</v>
@@ -985,19 +985,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1.674700183943275</v>
+        <v>2.343494150586636</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>1.704469904945673</v>
+        <v>2.385152453190655</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>1.676745166674422</v>
+        <v>2.346355800160955</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>1.69191796099463</v>
+        <v>2.367587872073516</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1.701856994641966</v>
+        <v>2.38149607333744</v>
       </c>
     </row>
     <row r="7">
@@ -1007,19 +1007,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5.099601325768251</v>
+        <v>5.099601325768182</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>5.138073760128728</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>5.884758195642447</v>
+        <v>5.88475819564244</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>6.297761850587959</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>6.551976629698161</v>
+        <v>6.551976629698165</v>
       </c>
     </row>
     <row r="8">
@@ -1051,19 +1051,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0.8055408769822704</v>
+        <v>2.599182845696212</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.7507291902940787</v>
+        <v>2.410129527017159</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.8003280765068828</v>
+        <v>2.581874243776133</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.7821672214605995</v>
+        <v>2.52028729842289</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0.8729301480665801</v>
+        <v>2.788155785203608</v>
       </c>
     </row>
     <row r="10">
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>3.460426177941363</v>
+        <v>3.870832167167569</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>3.128512170647415</v>
+        <v>3.518525984808759</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3.185565253129752</v>
+        <v>3.594091386589048</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3.068698653996409</v>
+        <v>3.470996985336605</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>3.014336008851963</v>
+        <v>3.446813461490714</v>
       </c>
     </row>
   </sheetData>
@@ -1197,19 +1197,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>6.22595921770089</v>
+        <v>8.647684382973296</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>6.336632800148852</v>
+        <v>8.801406914245572</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>6.233561760058678</v>
+        <v>8.658244103093434</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>6.289968990177773</v>
+        <v>8.736592178615814</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>6.326918898432972</v>
+        <v>8.787914574635099</v>
       </c>
     </row>
     <row r="7">
@@ -1219,19 +1219,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>49.08269257595933</v>
+        <v>49.08269257595922</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>51.34316205900213</v>
+        <v>51.34316205900203</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>61.73254233847679</v>
+        <v>61.73254233847681</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>65.87033548278535</v>
+        <v>65.87033548278512</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>73.4946295223331</v>
+        <v>73.49462952233317</v>
       </c>
     </row>
     <row r="8">
@@ -1263,19 +1263,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>10.4683017106039</v>
+        <v>30.30085032490308</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>9.759479175510052</v>
+        <v>28.08948488981295</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>10.1255790187319</v>
+        <v>28.69401070614894</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>8.957076297182045</v>
+        <v>25.62292108637144</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>11.05191889143878</v>
+        <v>30.98654883519867</v>
       </c>
     </row>
     <row r="10">
@@ -1285,19 +1285,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>19.58868738095201</v>
+        <v>23.29773301088059</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>18.29423408674348</v>
+        <v>21.76003072481006</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>19.74202767196945</v>
+        <v>23.24088001037809</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>19.88329097242071</v>
+        <v>23.06870230202525</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>20.99749619883145</v>
+        <v>24.73010046882513</v>
       </c>
     </row>
   </sheetData>
@@ -1377,7 +1377,7 @@
         <v>94.33775084566619</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>88.8717968238078</v>
+        <v>88.87179682380781</v>
       </c>
     </row>
     <row r="5">
@@ -1396,10 +1396,10 @@
         <v>74.59995103887134</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>58.78355940525261</v>
+        <v>58.78355940525262</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>66.59286994597188</v>
+        <v>66.59286994597186</v>
       </c>
     </row>
     <row r="6">
@@ -1415,13 +1415,13 @@
         <v>60.0935427865742</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>65.07612850013156</v>
+        <v>65.07612850013152</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>55.77213851154134</v>
+        <v>55.77213851154131</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>50.25085859008419</v>
+        <v>50.2508585900842</v>
       </c>
     </row>
     <row r="7">
@@ -1434,16 +1434,16 @@
         <v>38.63471126652675</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>45.88832516582504</v>
+        <v>45.88832516582501</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>44.53876283005371</v>
+        <v>44.53876283005372</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>39.67071028192908</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>40.13015546029065</v>
+        <v>40.13015546029064</v>
       </c>
     </row>
     <row r="8">
@@ -1453,13 +1453,13 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>50.91410095120624</v>
+        <v>50.91410095120618</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>50.47289416229471</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>47.84487225862026</v>
+        <v>47.84487225862024</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>42.70851717210358</v>
@@ -1497,16 +1497,16 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>64.0638344566235</v>
+        <v>64.06383445662348</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>65.80089442385021</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>65.14050815451024</v>
+        <v>65.14050815451021</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>57.08690847805255</v>
+        <v>57.08690847805254</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>59.14617154812704</v>
@@ -1589,7 +1589,7 @@
         <v>94.33775084566619</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>88.8717968238078</v>
+        <v>88.87179682380781</v>
       </c>
     </row>
     <row r="5">
@@ -1611,7 +1611,7 @@
         <v>60.48743069236139</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>67.14436369293645</v>
+        <v>67.14436369293644</v>
       </c>
     </row>
     <row r="6">
@@ -1627,13 +1627,13 @@
         <v>69.3002732134959</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>75.88299460484656</v>
+        <v>75.8829946048465</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>64.31680106259697</v>
+        <v>64.31680106259691</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>57.61546352765392</v>
+        <v>57.61546352765393</v>
       </c>
     </row>
     <row r="7">
@@ -1646,16 +1646,16 @@
         <v>54.84320614055069</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>58.37024562485339</v>
+        <v>58.37024562485334</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>56.51225593946253</v>
+        <v>56.51225593946255</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.34279731194104</v>
+        <v>49.34279731194102</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>49.20733907210177</v>
+        <v>49.20733907210176</v>
       </c>
     </row>
     <row r="8">
@@ -1665,13 +1665,13 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>69.80271586400637</v>
+        <v>69.80271586400629</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>69.1978258325949</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>65.59483446479334</v>
+        <v>65.59483446479332</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>58.55294375117026</v>
@@ -1712,13 +1712,13 @@
         <v>74.16244546297617</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>74.76991861026393</v>
+        <v>74.76991861026391</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>73.5239033540568</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>63.61292652972094</v>
+        <v>63.61292652972093</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>64.60692967954809</v>
@@ -1802,7 +1802,7 @@
         <v>2020</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>99.79425867013732</v>
@@ -1824,7 +1824,7 @@
         <v>2021</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>99.97719552064747</v>
@@ -1846,7 +1846,7 @@
         <v>2022</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>99.26847897567855</v>
@@ -1868,7 +1868,7 @@
         <v>2023</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>94.90719400972453</v>
@@ -1890,10 +1890,10 @@
         <v>2024</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>89.4082463016175</v>
+        <v>89.40824630161751</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>99.40000000000001</v>
@@ -1912,7 +1912,7 @@
         <v>2020</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>2.200000000000003</v>
+        <v>2.2</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>83.98969544323815</v>
@@ -1934,10 +1934,10 @@
         <v>2021</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>2.099999999999994</v>
+        <v>2.09999999999999</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>84.20375203717359</v>
+        <v>84.2037520371736</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>95.59999999999999</v>
@@ -1956,7 +1956,7 @@
         <v>2022</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>1.799999999999997</v>
+        <v>1.8</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>77.38584132663001</v>
@@ -1978,10 +1978,10 @@
         <v>2023</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>1.700000000000003</v>
+        <v>1.7</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>60.8525459681704</v>
+        <v>60.85254596817041</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>96.59999999999999</v>
@@ -2000,10 +2000,10 @@
         <v>2024</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>1.700000000000003</v>
+        <v>1.7</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>68.93671837057131</v>
+        <v>68.93671837057128</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>96.59999999999999</v>
@@ -2022,7 +2022,7 @@
         <v>2020</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>10.09999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="D14" s="11" t="n">
         <v>75.27843098172775</v>
@@ -2044,7 +2044,7 @@
         <v>2021</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>10.73999999999999</v>
+        <v>10.74</v>
       </c>
       <c r="D15" s="11" t="n">
         <v>71.37000330947055</v>
@@ -2069,7 +2069,7 @@
         <v>10.06</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>78.31062394721006</v>
+        <v>78.31062394721002</v>
       </c>
       <c r="E16" s="11" t="n">
         <v>83.09999999999999</v>
@@ -2091,7 +2091,7 @@
         <v>9.609999999999999</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>66.23769419422962</v>
+        <v>66.23769419422958</v>
       </c>
       <c r="E17" s="11" t="n">
         <v>84.2</v>
@@ -2113,7 +2113,7 @@
         <v>9.109999999999999</v>
       </c>
       <c r="D18" s="11" t="n">
-        <v>59.15345331381305</v>
+        <v>59.15345331381307</v>
       </c>
       <c r="E18" s="11" t="n">
         <v>84.95</v>
@@ -2157,7 +2157,7 @@
         <v>14.23</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>61.66956748531789</v>
+        <v>61.66956748531784</v>
       </c>
       <c r="E20" s="11" t="n">
         <v>74.41</v>
@@ -2179,7 +2179,7 @@
         <v>14.37</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>59.80765788915497</v>
+        <v>59.80765788915499</v>
       </c>
       <c r="E21" s="11" t="n">
         <v>74.47</v>
@@ -2201,7 +2201,7 @@
         <v>13.72</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>52.25330648304674</v>
+        <v>52.25330648304672</v>
       </c>
       <c r="E22" s="11" t="n">
         <v>75.92</v>
@@ -2245,7 +2245,7 @@
         <v>1.5</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>69.80271586400637</v>
+        <v>69.80271586400629</v>
       </c>
       <c r="E24" s="11" t="n">
         <v>72.94</v>
@@ -2264,7 +2264,7 @@
         <v>2021</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>0.9099999999999966</v>
+        <v>0.909999999999997</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>69.1978258325949</v>
@@ -2286,10 +2286,10 @@
         <v>2022</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>0.7399999999999949</v>
+        <v>0.739999999999995</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>65.59483446479334</v>
+        <v>65.59483446479332</v>
       </c>
       <c r="E26" s="11" t="n">
         <v>72.94</v>
@@ -2308,7 +2308,7 @@
         <v>2023</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>0.5900000000000034</v>
+        <v>0.590000000000003</v>
       </c>
       <c r="D27" s="11" t="n">
         <v>58.55294375117026</v>
@@ -2330,7 +2330,7 @@
         <v>2024</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0.4429999999999978</v>
+        <v>0.442999999999998</v>
       </c>
       <c r="D28" s="11" t="n">
         <v>51.80150021325011</v>
@@ -2352,7 +2352,7 @@
         <v>2020</v>
       </c>
       <c r="C29" s="11" t="n">
-        <v>5.599999999999994</v>
+        <v>5.59999999999999</v>
       </c>
       <c r="D29" s="11" t="n">
         <v>65.0397256367866</v>
@@ -2374,7 +2374,7 @@
         <v>2021</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>5.099999999999994</v>
+        <v>5.09999999999999</v>
       </c>
       <c r="D30" s="11" t="n">
         <v>68.52457386579727</v>
@@ -2396,7 +2396,7 @@
         <v>2022</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>4.799999999999997</v>
+        <v>4.8</v>
       </c>
       <c r="D31" s="11" t="n">
         <v>67.3441604373496</v>
@@ -2418,7 +2418,7 @@
         <v>2023</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>4.400000000000006</v>
+        <v>4.40000000000001</v>
       </c>
       <c r="D32" s="11" t="n">
         <v>54.69453004463444</v>

</xml_diff>

<commit_message>
feat: consolidar salidas regionales y visualizador SIEPAC
</commit_message>
<xml_diff>
--- a/data/processed/indicadores_SOC_SIEPAC.xlsx
+++ b/data/processed/indicadores_SOC_SIEPAC.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Metodologia" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SOC1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="SOC2_PROM" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="SOC2_POBRE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SOC2_VULNERABLE" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="SOC3_RURAL" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="SOC3_URB" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Datos_Base" sheetId="7" state="visible" r:id="rId7"/>
@@ -575,24 +575,24 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Cargo anual de electricidad ÷ Ingreso anual del hogar promedio × 100</t>
+          <t>Cargo anual medio residencial ÷ ingreso anual de referencia del hogar × 100</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Las dos series se resumen mediante promedio de países. Los insumos monetarios se conservan en el marco de cada país, por lo que no se construye una razón de sumas regional.</t>
+          <t>El agregado regional es la razón entre el gasto residencial proxy y el ingreso PROM proxy, ambos expandidos por clientes residenciales.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>SOC2_POBRE</t>
+          <t>SOC2_VULNERABLE</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SOC2 — Ingreso destinado a electricidad (quintil más pobre)</t>
+          <t>SOC2 — Ingreso destinado a electricidad (estrato vulnerable)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Cargo anual ÷ Ingreso anual del quintil de menores ingresos × 100</t>
+          <t>Cargo anual medio residencial ÷ ingreso anual del estrato vulnerable × 100</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Mismo criterio de agregación que SOC2 (hogar promedio).</t>
+          <t>El agregado regional usa clientes vulnerables proxy: 20 % en cinco países y 29.6 % en Nicaragua.</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -931,7 +931,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Fórmula: Cargo anual de electricidad ÷ Ingreso anual del hogar promedio × 100</t>
+          <t>Fórmula: Cargo anual medio residencial ÷ ingreso anual de referencia del hogar × 100</t>
         </is>
       </c>
     </row>
@@ -967,10 +967,10 @@
         <v>2.408128160981093</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>1.876613220735559</v>
+        <v>1.876613220735558</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>1.804921953715687</v>
+        <v>1.804921953715686</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>1.826309538261201</v>
@@ -1017,7 +1017,7 @@
         <v>2.346355800160955</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>2.367587872073516</v>
+        <v>2.367587872073515</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>2.38149607333744</v>
@@ -1030,19 +1030,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5.099601325768182</v>
+        <v>5.099601325768265</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>5.138073760128728</v>
+        <v>5.138073760128743</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>5.88475819564244</v>
+        <v>5.884758195642447</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>6.297761850587959</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>6.551976629698165</v>
+        <v>6.551976629698161</v>
       </c>
     </row>
     <row r="8">
@@ -1064,7 +1064,7 @@
         <v>6.085265483784632</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>5.314406722318093</v>
+        <v>5.18740633862105</v>
       </c>
     </row>
     <row r="9">
@@ -1074,19 +1074,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>2.599182845696212</v>
+        <v>1.083966087996522</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2.410129527017159</v>
+        <v>1.009601329371265</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>2.581874243776133</v>
+        <v>1.087310534384475</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2.52028729842289</v>
+        <v>1.066933189298826</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2.788155785203608</v>
+        <v>1.184511908743388</v>
       </c>
     </row>
     <row r="10">
@@ -1096,19 +1096,41 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>3.870832167167569</v>
+        <v>3.618296040884301</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>3.518525984808759</v>
+        <v>3.285104618534445</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3.594091386589048</v>
+        <v>3.344997435023773</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3.470996985336605</v>
+        <v>3.228771300482594</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>3.446813461490714</v>
+        <v>3.158372751464503</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Agregado regional (razón de sumas)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>2.139755107334277</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>2.004943223486199</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>2.045459401634776</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>2.029724011393092</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>2.112803729840648</v>
       </c>
     </row>
   </sheetData>
@@ -1122,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1136,14 +1158,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SOC2 — Ingreso destinado a electricidad (quintil más pobre) (%)</t>
+          <t>SOC2 — Ingreso destinado a electricidad (estrato vulnerable) (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Fórmula: Cargo anual ÷ Ingreso anual del quintil de menores ingresos × 100</t>
+          <t>Fórmula: Cargo anual medio residencial ÷ ingreso anual del estrato vulnerable × 100</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1198,7 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>21.71940305130531</v>
+        <v>21.7194030513053</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>15.74904272366592</v>
@@ -1198,7 +1220,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>7.2421669099111</v>
+        <v>7.242166909911102</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>7.554624109336666</v>
@@ -1223,7 +1245,7 @@
         <v>8.647684382973296</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>8.801406914245572</v>
+        <v>8.80140691424557</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>8.658244103093434</v>
@@ -1242,19 +1264,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>49.08269257595922</v>
+        <v>49.08269257595948</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>51.34316205900203</v>
+        <v>51.34316205900219</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>61.73254233847681</v>
+        <v>61.7325423384768</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>65.87033548278512</v>
+        <v>65.87033548278535</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>73.49462952233317</v>
+        <v>73.49462952233308</v>
       </c>
     </row>
     <row r="8">
@@ -1273,10 +1295,10 @@
         <v>18.52946062943986</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>15.9224764527489</v>
+        <v>15.92247645274891</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>13.90547645323327</v>
+        <v>13.57317203294221</v>
       </c>
     </row>
     <row r="9">
@@ -1286,19 +1308,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>30.30085032490308</v>
+        <v>13.4592451413831</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>28.08948488981295</v>
+        <v>12.54790187622861</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>28.69401070614894</v>
+        <v>12.88710061917378</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>25.62292108637144</v>
+        <v>11.56955680044087</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>30.98654883519867</v>
+        <v>14.0660786435457</v>
       </c>
     </row>
     <row r="10">
@@ -1308,19 +1330,41 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>23.29773301088059</v>
+        <v>20.4907988136273</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>21.76003072481006</v>
+        <v>19.1697668892127</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>23.24088001037809</v>
+        <v>20.60639499588222</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>23.06870230202525</v>
+        <v>20.72647492103686</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>24.73010046882513</v>
+        <v>21.85463803350111</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Agregado regional (razón de sumas)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>13.66266783904118</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>12.73577995477674</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>12.62876824655664</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>12.437856705476</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>12.94930321945495</v>
       </c>
     </row>
   </sheetData>
@@ -1802,7 +1846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:T33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1814,6 +1858,17 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1826,7 +1881,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Tasas y participaciones en %; población rural, urbana y total en habitantes. Los insumos monetarios de SOC2 (cargo medio e ingresos por grupo) permanecen en las hojas por país de SOCs.xlsx, en moneda local. Fuentes: SOCs.xlsx y Banco Mundial WDI (SP.RUR.TOTL y SP.URB.TOTL).</t>
+          <t>Tasas y participaciones en %; población rural, urbana y total en habitantes. SOC2 conserva cargo e ingresos anuales en USD, clientes residenciales y clientes vulnerables proxy. Fuentes: SOCs.xlsx, base única SOC2 del equipo y Banco Mundial WDI (SP.RUR.TOTL y SP.URB.TOTL).</t>
         </is>
       </c>
     </row>
@@ -1876,6 +1931,61 @@
           <t>poblacion_total_hab</t>
         </is>
       </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>clientes_residenciales</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>cargo_anual_usd</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>ingreso_prom_usd</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>ingreso_vulnerable_usd</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>proporcion_vulnerable</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>clientes_vulnerables_proxy</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>gasto_prom_proxy_usd</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>ingreso_prom_proxy_usd</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>gasto_vulnerable_proxy_usd</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>ingreso_vulnerable_proxy_usd</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>fuente_dato</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -1907,6 +2017,41 @@
       <c r="I4" s="12" t="n">
         <v>5034320</v>
       </c>
+      <c r="J4" s="11" t="n">
+        <v>1585123</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <v>399.355222321832</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>16583.63656854256</v>
+      </c>
+      <c r="M4" s="11" t="n">
+        <v>1838.702571053541</v>
+      </c>
+      <c r="N4" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O4" s="11" t="n">
+        <v>317024.6</v>
+      </c>
+      <c r="P4" s="11" t="n">
+        <v>633027148.0724493</v>
+      </c>
+      <c r="Q4" s="11" t="n">
+        <v>26287103748.43789</v>
+      </c>
+      <c r="R4" s="11" t="n">
+        <v>126605429.6144899</v>
+      </c>
+      <c r="S4" s="11" t="n">
+        <v>582913947.1072205</v>
+      </c>
+      <c r="T4" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1938,6 +2083,41 @@
       <c r="I5" s="12" t="n">
         <v>5059988</v>
       </c>
+      <c r="J5" s="11" t="n">
+        <v>1618851</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>340.6164517013918</v>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>18150.59426938725</v>
+      </c>
+      <c r="M5" s="11" t="n">
+        <v>2162.775590096984</v>
+      </c>
+      <c r="N5" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O5" s="11" t="n">
+        <v>323770.2</v>
+      </c>
+      <c r="P5" s="11" t="n">
+        <v>551407283.4532498</v>
+      </c>
+      <c r="Q5" s="11" t="n">
+        <v>29383107683.59182</v>
+      </c>
+      <c r="R5" s="11" t="n">
+        <v>110281456.69065</v>
+      </c>
+      <c r="S5" s="11" t="n">
+        <v>700242285.3608186</v>
+      </c>
+      <c r="T5" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1969,6 +2149,41 @@
       <c r="I6" s="12" t="n">
         <v>5081765</v>
       </c>
+      <c r="J6" s="11" t="n">
+        <v>1655881</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>327.3119659616946</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>18134.41103577231</v>
+      </c>
+      <c r="M6" s="11" t="n">
+        <v>2208.245646709976</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O6" s="11" t="n">
+        <v>331176.2</v>
+      </c>
+      <c r="P6" s="11" t="n">
+        <v>541989665.5086168</v>
+      </c>
+      <c r="Q6" s="11" t="n">
+        <v>30028426680.32568</v>
+      </c>
+      <c r="R6" s="11" t="n">
+        <v>108397933.1017234</v>
+      </c>
+      <c r="S6" s="11" t="n">
+        <v>731318401.9439526</v>
+      </c>
+      <c r="T6" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2000,6 +2215,41 @@
       <c r="I7" s="12" t="n">
         <v>5105525</v>
       </c>
+      <c r="J7" s="11" t="n">
+        <v>1689739</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>407.595162416541</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>22317.96712865036</v>
+      </c>
+      <c r="M7" s="11" t="n">
+        <v>2656.144278343377</v>
+      </c>
+      <c r="N7" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O7" s="11" t="n">
+        <v>337947.8</v>
+      </c>
+      <c r="P7" s="11" t="n">
+        <v>688729442.1465635</v>
+      </c>
+      <c r="Q7" s="11" t="n">
+        <v>37711539457.99854</v>
+      </c>
+      <c r="R7" s="11" t="n">
+        <v>137745888.4293127</v>
+      </c>
+      <c r="S7" s="11" t="n">
+        <v>897638115.348732</v>
+      </c>
+      <c r="T7" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2031,6 +2281,41 @@
       <c r="I8" s="12" t="n">
         <v>5129910</v>
       </c>
+      <c r="J8" s="11" t="n">
+        <v>1723337</v>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>468.1035768243329</v>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>24827.90392291269</v>
+      </c>
+      <c r="M8" s="11" t="n">
+        <v>3350.418276794394</v>
+      </c>
+      <c r="N8" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O8" s="11" t="n">
+        <v>344667.4</v>
+      </c>
+      <c r="P8" s="11" t="n">
+        <v>806700213.7737155</v>
+      </c>
+      <c r="Q8" s="11" t="n">
+        <v>42786845462.80059</v>
+      </c>
+      <c r="R8" s="11" t="n">
+        <v>161340042.7547431</v>
+      </c>
+      <c r="S8" s="11" t="n">
+        <v>1154779956.375204</v>
+      </c>
+      <c r="T8" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2062,6 +2347,41 @@
       <c r="I9" s="12" t="n">
         <v>6234673</v>
       </c>
+      <c r="J9" s="11" t="n">
+        <v>1762102</v>
+      </c>
+      <c r="K9" s="11" t="n">
+        <v>204.1552367570096</v>
+      </c>
+      <c r="L9" s="11" t="n">
+        <v>9894.55500000008</v>
+      </c>
+      <c r="M9" s="11" t="n">
+        <v>2818.979999999967</v>
+      </c>
+      <c r="N9" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O9" s="11" t="n">
+        <v>352420.4</v>
+      </c>
+      <c r="P9" s="11" t="n">
+        <v>359742351.0000001</v>
+      </c>
+      <c r="Q9" s="11" t="n">
+        <v>17435215154.61014</v>
+      </c>
+      <c r="R9" s="11" t="n">
+        <v>71948470.20000002</v>
+      </c>
+      <c r="S9" s="11" t="n">
+        <v>993466059.1919883</v>
+      </c>
+      <c r="T9" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -2093,6 +2413,41 @@
       <c r="I10" s="12" t="n">
         <v>6255782</v>
       </c>
+      <c r="J10" s="11" t="n">
+        <v>1816530</v>
+      </c>
+      <c r="K10" s="11" t="n">
+        <v>220.9727551980975</v>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>10879.11</v>
+      </c>
+      <c r="M10" s="11" t="n">
+        <v>2925</v>
+      </c>
+      <c r="N10" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O10" s="11" t="n">
+        <v>363306</v>
+      </c>
+      <c r="P10" s="11" t="n">
+        <v>401403639</v>
+      </c>
+      <c r="Q10" s="11" t="n">
+        <v>19762229688.3</v>
+      </c>
+      <c r="R10" s="11" t="n">
+        <v>80280727.8</v>
+      </c>
+      <c r="S10" s="11" t="n">
+        <v>1062670050</v>
+      </c>
+      <c r="T10" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -2124,6 +2479,41 @@
       <c r="I11" s="12" t="n">
         <v>6280319</v>
       </c>
+      <c r="J11" s="11" t="n">
+        <v>1864350</v>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>217.3444450559176</v>
+      </c>
+      <c r="L11" s="11" t="n">
+        <v>11653.65</v>
+      </c>
+      <c r="M11" s="11" t="n">
+        <v>3101.04</v>
+      </c>
+      <c r="N11" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O11" s="11" t="n">
+        <v>372870</v>
+      </c>
+      <c r="P11" s="11" t="n">
+        <v>405206116.14</v>
+      </c>
+      <c r="Q11" s="11" t="n">
+        <v>21726482377.5</v>
+      </c>
+      <c r="R11" s="11" t="n">
+        <v>81041223.22799999</v>
+      </c>
+      <c r="S11" s="11" t="n">
+        <v>1156284784.8</v>
+      </c>
+      <c r="T11" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2155,6 +2545,41 @@
       <c r="I12" s="12" t="n">
         <v>6309624</v>
       </c>
+      <c r="J12" s="11" t="n">
+        <v>1910891</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <v>230.2534758214885</v>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>13318.92</v>
+      </c>
+      <c r="M12" s="11" t="n">
+        <v>3330</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O12" s="11" t="n">
+        <v>382178.2</v>
+      </c>
+      <c r="P12" s="11" t="n">
+        <v>439989294.666</v>
+      </c>
+      <c r="Q12" s="11" t="n">
+        <v>25451004357.72</v>
+      </c>
+      <c r="R12" s="11" t="n">
+        <v>87997858.9332</v>
+      </c>
+      <c r="S12" s="11" t="n">
+        <v>1272653406</v>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2186,6 +2611,41 @@
       <c r="I13" s="12" t="n">
         <v>6338193</v>
       </c>
+      <c r="J13" s="11" t="n">
+        <v>1961053</v>
+      </c>
+      <c r="K13" s="11" t="n">
+        <v>239.6859915433188</v>
+      </c>
+      <c r="L13" s="11" t="n">
+        <v>13622.76</v>
+      </c>
+      <c r="M13" s="11" t="n">
+        <v>3313.08</v>
+      </c>
+      <c r="N13" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O13" s="11" t="n">
+        <v>392210.6</v>
+      </c>
+      <c r="P13" s="11" t="n">
+        <v>470036932.774</v>
+      </c>
+      <c r="Q13" s="11" t="n">
+        <v>26714954366.28</v>
+      </c>
+      <c r="R13" s="11" t="n">
+        <v>94007386.5548</v>
+      </c>
+      <c r="S13" s="11" t="n">
+        <v>1299425094.648</v>
+      </c>
+      <c r="T13" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -2217,6 +2677,41 @@
       <c r="I14" s="12" t="n">
         <v>17357325</v>
       </c>
+      <c r="J14" s="11" t="n">
+        <v>3454999</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>188.1418965966367</v>
+      </c>
+      <c r="L14" s="11" t="n">
+        <v>8028.263972817685</v>
+      </c>
+      <c r="M14" s="11" t="n">
+        <v>2175.633247752142</v>
+      </c>
+      <c r="N14" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O14" s="11" t="n">
+        <v>690999.8</v>
+      </c>
+      <c r="P14" s="11" t="n">
+        <v>650030064.5994831</v>
+      </c>
+      <c r="Q14" s="11" t="n">
+        <v>27737643997.82113</v>
+      </c>
+      <c r="R14" s="11" t="n">
+        <v>130006012.9198966</v>
+      </c>
+      <c r="S14" s="11" t="n">
+        <v>1503362139.070081</v>
+      </c>
+      <c r="T14" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -2248,6 +2743,41 @@
       <c r="I15" s="12" t="n">
         <v>17598650</v>
       </c>
+      <c r="J15" s="11" t="n">
+        <v>3530523</v>
+      </c>
+      <c r="K15" s="11" t="n">
+        <v>197.0467376482599</v>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>8261.389639252095</v>
+      </c>
+      <c r="M15" s="11" t="n">
+        <v>2238.809539976259</v>
+      </c>
+      <c r="N15" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O15" s="11" t="n">
+        <v>706104.6000000001</v>
+      </c>
+      <c r="P15" s="11" t="n">
+        <v>695678039.3421476</v>
+      </c>
+      <c r="Q15" s="11" t="n">
+        <v>29167026133.34122</v>
+      </c>
+      <c r="R15" s="11" t="n">
+        <v>139135607.8684295</v>
+      </c>
+      <c r="S15" s="11" t="n">
+        <v>1580833714.701121</v>
+      </c>
+      <c r="T15" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -2279,6 +2809,41 @@
       <c r="I16" s="12" t="n">
         <v>17847877</v>
       </c>
+      <c r="J16" s="11" t="n">
+        <v>3696152</v>
+      </c>
+      <c r="K16" s="11" t="n">
+        <v>211.3218733325677</v>
+      </c>
+      <c r="L16" s="11" t="n">
+        <v>9006.386555614094</v>
+      </c>
+      <c r="M16" s="11" t="n">
+        <v>2440.701264787236</v>
+      </c>
+      <c r="N16" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O16" s="11" t="n">
+        <v>739230.4</v>
+      </c>
+      <c r="P16" s="11" t="n">
+        <v>781077764.761917</v>
+      </c>
+      <c r="Q16" s="11" t="n">
+        <v>33288973680.30614</v>
+      </c>
+      <c r="R16" s="11" t="n">
+        <v>156215552.9523834</v>
+      </c>
+      <c r="S16" s="11" t="n">
+        <v>1804240572.249174</v>
+      </c>
+      <c r="T16" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -2310,6 +2875,41 @@
       <c r="I17" s="12" t="n">
         <v>18124838</v>
       </c>
+      <c r="J17" s="11" t="n">
+        <v>3794182</v>
+      </c>
+      <c r="K17" s="11" t="n">
+        <v>219.7652830193671</v>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>9282.243992359125</v>
+      </c>
+      <c r="M17" s="11" t="n">
+        <v>2515.457726838586</v>
+      </c>
+      <c r="N17" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O17" s="11" t="n">
+        <v>758836.4</v>
+      </c>
+      <c r="P17" s="11" t="n">
+        <v>833829481.0569882</v>
+      </c>
+      <c r="Q17" s="11" t="n">
+        <v>35218523075.41713</v>
+      </c>
+      <c r="R17" s="11" t="n">
+        <v>166765896.2113976</v>
+      </c>
+      <c r="S17" s="11" t="n">
+        <v>1908820885.786376</v>
+      </c>
+      <c r="T17" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -2341,6 +2941,41 @@
       <c r="I18" s="12" t="n">
         <v>18406359</v>
       </c>
+      <c r="J18" s="11" t="n">
+        <v>3847200</v>
+      </c>
+      <c r="K18" s="11" t="n">
+        <v>226.7780543100074</v>
+      </c>
+      <c r="L18" s="11" t="n">
+        <v>9522.503809640952</v>
+      </c>
+      <c r="M18" s="11" t="n">
+        <v>2580.567350581283</v>
+      </c>
+      <c r="N18" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O18" s="11" t="n">
+        <v>769440</v>
+      </c>
+      <c r="P18" s="11" t="n">
+        <v>872460530.5414606</v>
+      </c>
+      <c r="Q18" s="11" t="n">
+        <v>36634976656.45067</v>
+      </c>
+      <c r="R18" s="11" t="n">
+        <v>174492106.1082921</v>
+      </c>
+      <c r="S18" s="11" t="n">
+        <v>1985591742.231262</v>
+      </c>
+      <c r="T18" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -2372,6 +3007,41 @@
       <c r="I19" s="12" t="n">
         <v>10119640</v>
       </c>
+      <c r="J19" s="11" t="n">
+        <v>1752555</v>
+      </c>
+      <c r="K19" s="11" t="n">
+        <v>280.3666581829493</v>
+      </c>
+      <c r="L19" s="11" t="n">
+        <v>5497.815226579728</v>
+      </c>
+      <c r="M19" s="11" t="n">
+        <v>571.2128725396615</v>
+      </c>
+      <c r="N19" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O19" s="11" t="n">
+        <v>350511</v>
+      </c>
+      <c r="P19" s="11" t="n">
+        <v>491357988.6318188</v>
+      </c>
+      <c r="Q19" s="11" t="n">
+        <v>9635223564.418436</v>
+      </c>
+      <c r="R19" s="11" t="n">
+        <v>98271597.72636376</v>
+      </c>
+      <c r="S19" s="11" t="n">
+        <v>200216395.1667493</v>
+      </c>
+      <c r="T19" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -2403,6 +3073,41 @@
       <c r="I20" s="12" t="n">
         <v>10289877</v>
       </c>
+      <c r="J20" s="11" t="n">
+        <v>1790787</v>
+      </c>
+      <c r="K20" s="11" t="n">
+        <v>301.054372544966</v>
+      </c>
+      <c r="L20" s="11" t="n">
+        <v>5859.284755332562</v>
+      </c>
+      <c r="M20" s="11" t="n">
+        <v>586.357287848774</v>
+      </c>
+      <c r="N20" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O20" s="11" t="n">
+        <v>358157.4</v>
+      </c>
+      <c r="P20" s="11" t="n">
+        <v>539124256.646682</v>
+      </c>
+      <c r="Q20" s="11" t="n">
+        <v>10492730969.14773</v>
+      </c>
+      <c r="R20" s="11" t="n">
+        <v>107824851.3293364</v>
+      </c>
+      <c r="S20" s="11" t="n">
+        <v>210008201.6869685</v>
+      </c>
+      <c r="T20" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -2434,6 +3139,41 @@
       <c r="I21" s="12" t="n">
         <v>10463872</v>
       </c>
+      <c r="J21" s="11" t="n">
+        <v>1796949</v>
+      </c>
+      <c r="K21" s="11" t="n">
+        <v>355.0800228926764</v>
+      </c>
+      <c r="L21" s="11" t="n">
+        <v>6033.893170931076</v>
+      </c>
+      <c r="M21" s="11" t="n">
+        <v>575.1909923712332</v>
+      </c>
+      <c r="N21" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O21" s="11" t="n">
+        <v>359389.8</v>
+      </c>
+      <c r="P21" s="11" t="n">
+        <v>638060692.056972</v>
+      </c>
+      <c r="Q21" s="11" t="n">
+        <v>10842598299.61143</v>
+      </c>
+      <c r="R21" s="11" t="n">
+        <v>127612138.4113944</v>
+      </c>
+      <c r="S21" s="11" t="n">
+        <v>206717775.710099</v>
+      </c>
+      <c r="T21" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -2465,6 +3205,41 @@
       <c r="I22" s="12" t="n">
         <v>10644851</v>
       </c>
+      <c r="J22" s="11" t="n">
+        <v>1819474</v>
+      </c>
+      <c r="K22" s="11" t="n">
+        <v>382.7839568587768</v>
+      </c>
+      <c r="L22" s="11" t="n">
+        <v>6078.095138244074</v>
+      </c>
+      <c r="M22" s="11" t="n">
+        <v>581.1173634584177</v>
+      </c>
+      <c r="N22" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O22" s="11" t="n">
+        <v>363894.8000000001</v>
+      </c>
+      <c r="P22" s="11" t="n">
+        <v>696465457.1216661</v>
+      </c>
+      <c r="Q22" s="11" t="n">
+        <v>11058936073.5615</v>
+      </c>
+      <c r="R22" s="11" t="n">
+        <v>139293091.4243332</v>
+      </c>
+      <c r="S22" s="11" t="n">
+        <v>211465586.7522282</v>
+      </c>
+      <c r="T22" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -2496,6 +3271,41 @@
       <c r="I23" s="12" t="n">
         <v>10825703</v>
       </c>
+      <c r="J23" s="11" t="n">
+        <v>1900045</v>
+      </c>
+      <c r="K23" s="11" t="n">
+        <v>421.0610932475884</v>
+      </c>
+      <c r="L23" s="11" t="n">
+        <v>6426.474284707361</v>
+      </c>
+      <c r="M23" s="11" t="n">
+        <v>572.9140972397704</v>
+      </c>
+      <c r="N23" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O23" s="11" t="n">
+        <v>380009</v>
+      </c>
+      <c r="P23" s="11" t="n">
+        <v>800035024.9196141</v>
+      </c>
+      <c r="Q23" s="11" t="n">
+        <v>12210590332.2868</v>
+      </c>
+      <c r="R23" s="11" t="n">
+        <v>160007004.9839228</v>
+      </c>
+      <c r="S23" s="11" t="n">
+        <v>217712513.1779879</v>
+      </c>
+      <c r="T23" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -2527,6 +3337,41 @@
       <c r="I24" s="12" t="n">
         <v>6565267</v>
       </c>
+      <c r="J24" s="11" t="n">
+        <v>1155606</v>
+      </c>
+      <c r="K24" s="11" t="n">
+        <v>167.780178012512</v>
+      </c>
+      <c r="L24" s="11" t="n">
+        <v>1926.01115338162</v>
+      </c>
+      <c r="M24" s="11" t="n">
+        <v>736.0845674878655</v>
+      </c>
+      <c r="N24" s="11" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="O24" s="11" t="n">
+        <v>342059.376</v>
+      </c>
+      <c r="P24" s="11" t="n">
+        <v>193887780.392327</v>
+      </c>
+      <c r="Q24" s="11" t="n">
+        <v>2225710044.914721</v>
+      </c>
+      <c r="R24" s="11" t="n">
+        <v>57390782.99612879</v>
+      </c>
+      <c r="S24" s="11" t="n">
+        <v>251784627.8381292</v>
+      </c>
+      <c r="T24" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -2558,6 +3403,41 @@
       <c r="I25" s="12" t="n">
         <v>6644741</v>
       </c>
+      <c r="J25" s="11" t="n">
+        <v>1209264</v>
+      </c>
+      <c r="K25" s="11" t="n">
+        <v>141.0668715343602</v>
+      </c>
+      <c r="L25" s="11" t="n">
+        <v>1940.391472232593</v>
+      </c>
+      <c r="M25" s="11" t="n">
+        <v>741.5804498783546</v>
+      </c>
+      <c r="N25" s="11" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="O25" s="11" t="n">
+        <v>357942.144</v>
+      </c>
+      <c r="P25" s="11" t="n">
+        <v>170587089.3391265</v>
+      </c>
+      <c r="Q25" s="11" t="n">
+        <v>2346445553.277874</v>
+      </c>
+      <c r="R25" s="11" t="n">
+        <v>50493778.44438145</v>
+      </c>
+      <c r="S25" s="11" t="n">
+        <v>265442896.1779428</v>
+      </c>
+      <c r="T25" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -2589,6 +3469,41 @@
       <c r="I26" s="12" t="n">
         <v>6730654</v>
       </c>
+      <c r="J26" s="11" t="n">
+        <v>1225848</v>
+      </c>
+      <c r="K26" s="11" t="n">
+        <v>144.1716088953862</v>
+      </c>
+      <c r="L26" s="11" t="n">
+        <v>2035.860670232292</v>
+      </c>
+      <c r="M26" s="11" t="n">
+        <v>778.0669485129229</v>
+      </c>
+      <c r="N26" s="11" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="O26" s="11" t="n">
+        <v>362851.008</v>
+      </c>
+      <c r="P26" s="11" t="n">
+        <v>176732478.4211913</v>
+      </c>
+      <c r="Q26" s="11" t="n">
+        <v>2495655730.882915</v>
+      </c>
+      <c r="R26" s="11" t="n">
+        <v>52312813.61267263</v>
+      </c>
+      <c r="S26" s="11" t="n">
+        <v>282322376.5593981</v>
+      </c>
+      <c r="T26" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -2620,6 +3535,41 @@
       <c r="I27" s="12" t="n">
         <v>6823613</v>
       </c>
+      <c r="J27" s="11" t="n">
+        <v>1265190</v>
+      </c>
+      <c r="K27" s="11" t="n">
+        <v>134.448944668347</v>
+      </c>
+      <c r="L27" s="11" t="n">
+        <v>2209.417896829847</v>
+      </c>
+      <c r="M27" s="11" t="n">
+        <v>844.3971957963569</v>
+      </c>
+      <c r="N27" s="11" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="O27" s="11" t="n">
+        <v>374496.24</v>
+      </c>
+      <c r="P27" s="11" t="n">
+        <v>170103460.3049459</v>
+      </c>
+      <c r="Q27" s="11" t="n">
+        <v>2795333428.890153</v>
+      </c>
+      <c r="R27" s="11" t="n">
+        <v>50350624.250264</v>
+      </c>
+      <c r="S27" s="11" t="n">
+        <v>316223574.8922794</v>
+      </c>
+      <c r="T27" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -2651,6 +3601,41 @@
       <c r="I28" s="12" t="n">
         <v>6916140</v>
       </c>
+      <c r="J28" s="11" t="n">
+        <v>1299136.2</v>
+      </c>
+      <c r="K28" s="11" t="n">
+        <v>125.4716853385493</v>
+      </c>
+      <c r="L28" s="11" t="n">
+        <v>2418.774955113753</v>
+      </c>
+      <c r="M28" s="11" t="n">
+        <v>924.4094529563788</v>
+      </c>
+      <c r="N28" s="11" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="O28" s="11" t="n">
+        <v>384544.3152</v>
+      </c>
+      <c r="P28" s="11" t="n">
+        <v>163004808.4983186</v>
+      </c>
+      <c r="Q28" s="11" t="n">
+        <v>3142318103.841651</v>
+      </c>
+      <c r="R28" s="11" t="n">
+        <v>48249423.3155023</v>
+      </c>
+      <c r="S28" s="11" t="n">
+        <v>355476400.0515172</v>
+      </c>
+      <c r="T28" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -2682,6 +3667,41 @@
       <c r="I29" s="12" t="n">
         <v>4293261</v>
       </c>
+      <c r="J29" s="11" t="n">
+        <v>1061959.5</v>
+      </c>
+      <c r="K29" s="11" t="n">
+        <v>527.0748131166961</v>
+      </c>
+      <c r="L29" s="11" t="n">
+        <v>48624.65892183772</v>
+      </c>
+      <c r="M29" s="11" t="n">
+        <v>3916.080044460301</v>
+      </c>
+      <c r="N29" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O29" s="11" t="n">
+        <v>212391.9</v>
+      </c>
+      <c r="P29" s="11" t="n">
+        <v>559732105</v>
+      </c>
+      <c r="Q29" s="11" t="n">
+        <v>51637418476.30532</v>
+      </c>
+      <c r="R29" s="11" t="n">
+        <v>111946421</v>
+      </c>
+      <c r="S29" s="11" t="n">
+        <v>831743681.1950079</v>
+      </c>
+      <c r="T29" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -2713,6 +3733,41 @@
       <c r="I30" s="12" t="n">
         <v>4345405</v>
       </c>
+      <c r="J30" s="11" t="n">
+        <v>1095404</v>
+      </c>
+      <c r="K30" s="11" t="n">
+        <v>491.3858813734476</v>
+      </c>
+      <c r="L30" s="11" t="n">
+        <v>48671.27915525436</v>
+      </c>
+      <c r="M30" s="11" t="n">
+        <v>3916.080044460297</v>
+      </c>
+      <c r="N30" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O30" s="11" t="n">
+        <v>219080.8</v>
+      </c>
+      <c r="P30" s="11" t="n">
+        <v>538266060</v>
+      </c>
+      <c r="Q30" s="11" t="n">
+        <v>53314713871.78224</v>
+      </c>
+      <c r="R30" s="11" t="n">
+        <v>107653212</v>
+      </c>
+      <c r="S30" s="11" t="n">
+        <v>857937949.0043975</v>
+      </c>
+      <c r="T30" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -2744,6 +3799,41 @@
       <c r="I31" s="12" t="n">
         <v>4400773</v>
       </c>
+      <c r="J31" s="11" t="n">
+        <v>1139094</v>
+      </c>
+      <c r="K31" s="11" t="n">
+        <v>528.7010466212622</v>
+      </c>
+      <c r="L31" s="11" t="n">
+        <v>48624.65964431762</v>
+      </c>
+      <c r="M31" s="11" t="n">
+        <v>4102.560088920593</v>
+      </c>
+      <c r="N31" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O31" s="11" t="n">
+        <v>227818.8</v>
+      </c>
+      <c r="P31" s="11" t="n">
+        <v>602240190</v>
+      </c>
+      <c r="Q31" s="11" t="n">
+        <v>55388058052.88433</v>
+      </c>
+      <c r="R31" s="11" t="n">
+        <v>120448038</v>
+      </c>
+      <c r="S31" s="11" t="n">
+        <v>934640316.3857828</v>
+      </c>
+      <c r="T31" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -2775,6 +3865,41 @@
       <c r="I32" s="12" t="n">
         <v>4458759</v>
       </c>
+      <c r="J32" s="11" t="n">
+        <v>1179331</v>
+      </c>
+      <c r="K32" s="11" t="n">
+        <v>517.7978362308801</v>
+      </c>
+      <c r="L32" s="11" t="n">
+        <v>48531.42084474564</v>
+      </c>
+      <c r="M32" s="11" t="n">
+        <v>4475.520066690446</v>
+      </c>
+      <c r="N32" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O32" s="11" t="n">
+        <v>235866.2</v>
+      </c>
+      <c r="P32" s="11" t="n">
+        <v>610655040</v>
+      </c>
+      <c r="Q32" s="11" t="n">
+        <v>57234609076.25472</v>
+      </c>
+      <c r="R32" s="11" t="n">
+        <v>122131008</v>
+      </c>
+      <c r="S32" s="11" t="n">
+        <v>1055623911.154022</v>
+      </c>
+      <c r="T32" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2805,6 +3930,41 @@
       </c>
       <c r="I33" s="12" t="n">
         <v>4515577</v>
+      </c>
+      <c r="J33" s="11" t="n">
+        <v>1205983</v>
+      </c>
+      <c r="K33" s="11" t="n">
+        <v>577.069328506289</v>
+      </c>
+      <c r="L33" s="11" t="n">
+        <v>48717.90011115075</v>
+      </c>
+      <c r="M33" s="11" t="n">
+        <v>4102.560088920593</v>
+      </c>
+      <c r="N33" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O33" s="11" t="n">
+        <v>241196.6</v>
+      </c>
+      <c r="P33" s="11" t="n">
+        <v>695935800</v>
+      </c>
+      <c r="Q33" s="11" t="n">
+        <v>58752959329.74591</v>
+      </c>
+      <c r="R33" s="11" t="n">
+        <v>139187160</v>
+      </c>
+      <c r="S33" s="11" t="n">
+        <v>989523544.7433448</v>
+      </c>
+      <c r="T33" s="11" t="inlineStr">
+        <is>
+          <t>equipo_SOC2_base_unica</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>